<commit_message>
feat: added protocol documentation, standardized site layouts, and update project tracking status
</commit_message>
<xml_diff>
--- a/ROADMAP-HUB.xlsx
+++ b/ROADMAP-HUB.xlsx
@@ -748,6 +748,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>1.1</t>
@@ -778,8 +783,18 @@
           <t>status, hormoni, ultima_actualizare, versiune</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
           <t>1.2</t>
@@ -810,8 +825,18 @@
           <t>dificultate, categorie, status, dată</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>1.3</t>
@@ -840,6 +865,11 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>Update manual la fiecare release</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1921,6 +1951,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>S2</t>
@@ -1944,6 +1979,11 @@
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Metadata + badge layout + CHANGELOG</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: added dynamic protocol filtering, printable laboratory checklist, and glossary script, more in status oage
</commit_message>
<xml_diff>
--- a/ROADMAP-HUB.xlsx
+++ b/ROADMAP-HUB.xlsx
@@ -874,6 +874,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>1.4</t>
@@ -904,8 +909,18 @@
           <t>după categorie, dificultate, hormoni</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>1.5</t>
@@ -936,8 +951,18 @@
           <t>checkbox-uri pentru laborator</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>1.6</t>
@@ -968,8 +993,18 @@
           <t>două intrări separate în glossary.js</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>1.7</t>
@@ -998,6 +1033,11 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>nu card mort fără acțiune</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -1988,6 +2028,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>S3</t>
@@ -2011,6 +2056,11 @@
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Index filtrabil + checklist print + glossary fix</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: optimized the comprehensive library of plant protocols, research resources, and technical guidance documentation
</commit_message>
<xml_diff>
--- a/ROADMAP-HUB.xlsx
+++ b/ROADMAP-HUB.xlsx
@@ -2226,6 +2226,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>S7</t>
@@ -2249,6 +2254,11 @@
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>feed.xml + status.md + polish SEO descriptions</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>

</xml_diff>